<commit_message>
docs: sync BOM notes in English README
</commit_message>
<xml_diff>
--- a/Docs/BOM.xlsx
+++ b/Docs/BOM.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94ED6EBD-0B56-4490-976A-87698BE20B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C43E70-B362-434B-B67E-556662BCF52D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="243">
   <si>
     <t>No.</t>
   </si>
@@ -606,9 +606,6 @@
   </si>
   <si>
     <t>46</t>
-  </si>
-  <si>
-    <t>ACS712ELCTR-30A-T-JSM</t>
   </si>
   <si>
     <t>U6</t>
@@ -742,6 +739,14 @@
   </si>
   <si>
     <t>1:200互感器！！不要买错成1:100</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ACS712ELCTR-20A-T-JSM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>20A版本！！不要买错成30A版的！！</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1138,7 +1143,9 @@
   <dimension ref="A1:J55"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="10" width="20" customWidth="1"/>
+    <col min="1" max="5" width="20" customWidth="1"/>
+    <col min="6" max="6" width="33" customWidth="1"/>
+    <col min="7" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
@@ -2621,25 +2628,25 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
+        <v>241</v>
+      </c>
+      <c r="D47" t="s">
         <v>197</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>198</v>
       </c>
-      <c r="E47" t="s">
+      <c r="F47" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G47" t="s">
+        <v>241</v>
+      </c>
+      <c r="H47" t="s">
         <v>199</v>
       </c>
-      <c r="F47" t="s">
-        <v>14</v>
-      </c>
-      <c r="G47" t="s">
-        <v>197</v>
-      </c>
-      <c r="H47" t="s">
+      <c r="I47" t="s">
         <v>200</v>
-      </c>
-      <c r="I47" t="s">
-        <v>201</v>
       </c>
       <c r="J47" t="s">
         <v>37</v>
@@ -2647,31 +2654,31 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B48">
         <v>2</v>
       </c>
       <c r="C48" t="s">
+        <v>202</v>
+      </c>
+      <c r="D48" t="s">
         <v>203</v>
       </c>
-      <c r="D48" t="s">
+      <c r="E48" t="s">
         <v>204</v>
       </c>
-      <c r="E48" t="s">
-        <v>205</v>
-      </c>
       <c r="F48" t="s">
         <v>14</v>
       </c>
       <c r="G48" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H48" t="s">
         <v>98</v>
       </c>
       <c r="I48" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="J48" t="s">
         <v>37</v>
@@ -2679,28 +2686,28 @@
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>206</v>
+      </c>
+      <c r="B49">
+        <v>1</v>
+      </c>
+      <c r="C49" t="s">
+        <v>239</v>
+      </c>
+      <c r="D49" t="s">
         <v>207</v>
       </c>
-      <c r="B49">
-        <v>1</v>
-      </c>
-      <c r="C49" t="s">
+      <c r="E49" t="s">
+        <v>208</v>
+      </c>
+      <c r="F49" s="1" t="s">
         <v>240</v>
       </c>
-      <c r="D49" t="s">
-        <v>208</v>
-      </c>
-      <c r="E49" t="s">
+      <c r="H49" t="s">
         <v>209</v>
       </c>
-      <c r="F49" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="H49" t="s">
+      <c r="I49" t="s">
         <v>210</v>
-      </c>
-      <c r="I49" t="s">
-        <v>211</v>
       </c>
       <c r="J49" t="s">
         <v>37</v>
@@ -2708,31 +2715,31 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>211</v>
+      </c>
+      <c r="B50">
+        <v>1</v>
+      </c>
+      <c r="C50" t="s">
         <v>212</v>
       </c>
-      <c r="B50">
-        <v>1</v>
-      </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>213</v>
       </c>
-      <c r="D50" t="s">
+      <c r="E50" t="s">
         <v>214</v>
       </c>
-      <c r="E50" t="s">
+      <c r="F50" t="s">
+        <v>14</v>
+      </c>
+      <c r="G50" t="s">
+        <v>212</v>
+      </c>
+      <c r="H50" t="s">
         <v>215</v>
       </c>
-      <c r="F50" t="s">
-        <v>14</v>
-      </c>
-      <c r="G50" t="s">
-        <v>213</v>
-      </c>
-      <c r="H50" t="s">
+      <c r="I50" t="s">
         <v>216</v>
-      </c>
-      <c r="I50" t="s">
-        <v>217</v>
       </c>
       <c r="J50" t="s">
         <v>37</v>
@@ -2740,19 +2747,19 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>217</v>
+      </c>
+      <c r="B51">
+        <v>1</v>
+      </c>
+      <c r="C51" t="s">
         <v>218</v>
       </c>
-      <c r="B51">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>219</v>
       </c>
-      <c r="D51" t="s">
+      <c r="E51" t="s">
         <v>220</v>
-      </c>
-      <c r="E51" t="s">
-        <v>221</v>
       </c>
       <c r="F51" t="s">
         <v>14</v>
@@ -2772,31 +2779,31 @@
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>221</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
+      </c>
+      <c r="C52" t="s">
         <v>222</v>
       </c>
-      <c r="B52">
-        <v>1</v>
-      </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>223</v>
       </c>
-      <c r="D52" t="s">
+      <c r="E52" t="s">
         <v>224</v>
       </c>
-      <c r="E52" t="s">
+      <c r="F52" t="s">
+        <v>14</v>
+      </c>
+      <c r="G52" t="s">
+        <v>222</v>
+      </c>
+      <c r="H52" t="s">
         <v>225</v>
       </c>
-      <c r="F52" t="s">
-        <v>14</v>
-      </c>
-      <c r="G52" t="s">
-        <v>223</v>
-      </c>
-      <c r="H52" t="s">
+      <c r="I52" t="s">
         <v>226</v>
-      </c>
-      <c r="I52" t="s">
-        <v>227</v>
       </c>
       <c r="J52" t="s">
         <v>37</v>
@@ -2804,31 +2811,31 @@
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B53">
         <v>2</v>
       </c>
       <c r="C53" t="s">
+        <v>228</v>
+      </c>
+      <c r="D53" t="s">
         <v>229</v>
       </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
         <v>230</v>
       </c>
-      <c r="E53" t="s">
-        <v>231</v>
-      </c>
       <c r="F53" t="s">
         <v>14</v>
       </c>
       <c r="G53" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H53" t="s">
         <v>98</v>
       </c>
       <c r="I53" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="J53" t="s">
         <v>37</v>
@@ -2836,31 +2843,31 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>232</v>
+      </c>
+      <c r="B54">
+        <v>1</v>
+      </c>
+      <c r="C54" t="s">
         <v>233</v>
       </c>
-      <c r="B54">
-        <v>1</v>
-      </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>234</v>
       </c>
-      <c r="D54" t="s">
+      <c r="E54" t="s">
         <v>235</v>
       </c>
-      <c r="E54" t="s">
+      <c r="F54" t="s">
+        <v>233</v>
+      </c>
+      <c r="G54" t="s">
         <v>236</v>
       </c>
-      <c r="F54" t="s">
-        <v>234</v>
-      </c>
-      <c r="G54" t="s">
+      <c r="H54" t="s">
         <v>237</v>
       </c>
-      <c r="H54" t="s">
+      <c r="I54" t="s">
         <v>238</v>
-      </c>
-      <c r="I54" t="s">
-        <v>239</v>
       </c>
       <c r="J54" t="s">
         <v>37</v>
@@ -2875,6 +2882,6 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>